<commit_message>
fix: correct swapped contract shares and dashboard wording; relabel revenue lost to churn
</commit_message>
<xml_diff>
--- a/Telco_Churn_Analysis.xlsx
+++ b/Telco_Churn_Analysis.xlsx
@@ -5,13 +5,13 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taofeeksalami/Desktop/Harjii/DAV_Portfolio/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taofeeksalami/Telco_Customer_Churn_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B7A61C-3CF8-134F-8319-DDBBA78DA0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="MKno8Rk8H3j9R42XnMw+0cJYymN9JmN8CmEIujZH0aKW3574fpr/rsIVHwELVCPliSOdVnIkew4dErdPTIs9BQ==" workbookSaltValue="XMxiKTKcD+NALzw573fuOQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16500" firstSheet="16" activeTab="24" xr2:uid="{B76D0E22-31AB-FB41-B59B-52BD901C65CA}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14500" firstSheet="20" activeTab="24" xr2:uid="{B76D0E22-31AB-FB41-B59B-52BD901C65CA}"/>
   </bookViews>
   <sheets>
     <sheet name="perfect_storm_churn" sheetId="15" r:id="rId1"/>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="112">
   <si>
     <t>No</t>
   </si>
@@ -381,13 +381,13 @@
     <t>tbl_AvgTenureByChurn</t>
   </si>
   <si>
-    <t>Monthly Revenue at Risk (£)</t>
+    <t>Monthly Revenue Lost to Churn (£)</t>
   </si>
   <si>
     <t>tbl_RevenueAtRisk</t>
   </si>
   <si>
-    <t>Revenue at Risk %</t>
+    <t>Revenue Lost to Churn (% of monthly charges)</t>
   </si>
   <si>
     <t>Avg Monthly Charge — Churned (£)</t>
@@ -453,10 +453,10 @@
     <t>High Risk</t>
   </si>
   <si>
-    <t>Revenue at Risk Summary</t>
+    <t>Revenue Lost to Churn Summary</t>
   </si>
   <si>
-    <t>Annualised Revenue at Risk (£)</t>
+    <t>Annualised Revenue Lost to Churn (£)</t>
   </si>
   <si>
     <t>Project 7 — KPI Framework</t>
@@ -469,6 +469,9 @@
   </si>
   <si>
     <t>Segment Descriptions</t>
+  </si>
+  <si>
+    <t>Revenue Lost to Churn (% of monthly charges)</t>
   </si>
 </sst>
 </file>
@@ -712,6 +715,8 @@
     <xf numFmtId="2" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -721,8 +726,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2378,10 +2381,10 @@
                   <c:v>55.02</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.07</c:v>
+                  <c:v>20.91</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.91</c:v>
+                  <c:v>24.07</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2490,10 +2493,10 @@
                   <c:v>56.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.58</c:v>
+                  <c:v>21.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.01</c:v>
+                  <c:v>22.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5141,10 +5144,10 @@
                   <c:v>55.02</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.07</c:v>
+                  <c:v>20.91</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.91</c:v>
+                  <c:v>24.07</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5256,10 +5259,10 @@
                   <c:v>56.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.58</c:v>
+                  <c:v>21.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.01</c:v>
+                  <c:v>22.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7155,10 +7158,10 @@
                   <c:v>55.02</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.07</c:v>
+                  <c:v>20.91</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.91</c:v>
+                  <c:v>24.07</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7267,10 +7270,10 @@
                   <c:v>56.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.58</c:v>
+                  <c:v>21.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.01</c:v>
+                  <c:v>22.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8293,7 +8296,7 @@
                 </a:solidFill>
                 <a:effectLst/>
               </a:rPr>
-              <a:t>Monthly Revenue at Risk vs Retained</a:t>
+              <a:t>Monthly Revenue Lost vs Retained</a:t>
             </a:r>
             <a:endParaRPr lang="en-GB" sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -24910,7 +24913,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Month-to-month contracts are the strongest churn driver (42.71%), with a churn rate 15× higher than two-year contracts.</a:t>
+            <a:t>• Month-to-month contracts have the highest churn rate (42.71%), 15× that of two-year contracts.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -24922,7 +24925,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Customer attrition is concentrated early, with 47.44% of churn occurring within the first 12 months.</a:t>
+            <a:t>• Churn is concentrated early: customers in their first 12 months churn at 47.44% and make up 55.5% of all churners.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -24934,7 +24937,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Electronic check customers are the highest-risk payment segment, with a churn rate of 45.29%—more than 3× that of automatic payment customers.</a:t>
+            <a:t>• Electronic check customers have the highest churn rate of any payment method (45.29%), about 3× that of automatic payment (15.2–16.7%).</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -25618,7 +25621,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>⚠ Early tenure churn</a:t>
+            <a:t>⚠ 0–12 month churn rate</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27010,7 +27013,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Customer Churn Puts £1.67M of Annual Revenue at Risk</a:t>
+            <a:t>Churned Customers Were Paying £1.67M a Year</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27290,7 +27293,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Month-to-month customers record the highest churn rate (42.7%) while also representing the largest share of monthly revenue exposure.</a:t>
+            <a:t>Month-to-month customers record the highest churn rate (42.7%) while also contributing the largest share of monthly revenue (56.4%).</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27545,7 +27548,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue at risk</a:t>
+            <a:t>Revenue lost to churn</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27997,7 +28000,7 @@
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>Monthly Revenue at Risk vs Retained</a:t>
+              <a:t>Monthly Revenue Lost vs Retained</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -28394,7 +28397,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Month-to-month contracts are the primary churn driver, with a churn rate of 42.71%—15× higher than two-year contracts.</a:t>
+            <a:t>• Month-to-month contracts have the highest churn rate, 42.71%—15× that of two-year contracts.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -28406,7 +28409,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Current churn represents a monthly revenue loss of £139K (30.5%), placing an estimated £1.67M in annual revenue at risk.</a:t>
+            <a:t>• Churned customers had been paying £139K a month (30.5% of monthly charges), about £1.67M a year.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -28418,7 +28421,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• A cohort of 814 high-risk customers is churning at 69.53%—more than three times the standard customer churn rate (20.92%).</a:t>
+            <a:t>• 814 customers fit the high-risk profile and churned at 69.53%, 3.3× the 20.92% rate for all others; 566 had already left.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -28646,7 +28649,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Target the 814 high-risk customers with personalised retention offers before renewal.</a:t>
+            <a:t>• Test the high-risk profile on active customers before using it to target offers.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -31066,7 +31069,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• The business is heavily exposed to month-to-month contracts, where 55% of customers generate 56% of total revenue.</a:t>
+              <a:t>• The business is heavily exposed to month-to-month contracts, where 55% of customers generate 56% of monthly revenue.</a:t>
             </a:r>
           </a:p>
           <a:p>
@@ -31090,7 +31093,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• The 814 high-risk customers are churning at 69.53%—more than three times the rate of the standard customer base (20.92%).</a:t>
+              <a:t>• The 814 customers in the high-risk profile churned at 69.53%, 3.3× the 20.92% rate for all others; 566 had already left.</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -31285,7 +31288,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• Implement proactive outreach for high-risk customers using early-warning indicators and personalised retention offers.</a:t>
+              <a:t>• Test the high-risk profile on active customers; if it holds, use it to prioritise outreach and retention offers.</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -33193,7 +33196,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue Stability Analysis — At Risk Revenue, Contract Value &amp; Customer LTV</a:t>
+            <a:t>Revenue Stability Analysis — Revenue Lost to Churn, Contract Value &amp; Customer LTV</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -33269,7 +33272,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue pillar · Total monthly charges £456K · 30.5% at risk · Annualised risk £1.67M</a:t>
+            <a:t>Revenue pillar · Total monthly charges £456K · 30.5% lost to churn · £1.67M a year</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -33496,7 +33499,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Monthly Revenue at Risk vs Retained</a:t>
+            <a:t>Monthly Revenue Lost vs Retained</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -33738,7 +33741,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• The business is losing its highest-value customers, with churned customers paying £13.17 more per month on average than retained customers.</a:t>
+              <a:t>• Churned customers were paying £13.17 more per month on average than retained customers (£74.44 vs £61.27).</a:t>
             </a:r>
           </a:p>
           <a:p>
@@ -34410,7 +34413,7 @@
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:pPr marL="0" indent="0" algn="l"/>
-            <a:t>30.50%</a:t>
+            <a:t>£139,131</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="3600" b="1">
             <a:solidFill>
@@ -34460,7 +34463,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue at risk</a:t>
+            <a:t>Revenue lost to churn</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -37123,10 +37126,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="58" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="56"/>
+      <c r="B1" s="58"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
@@ -37169,7 +37172,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="27" t="s">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="B5" s="29">
         <f>revenue_at_risk!D2</f>
@@ -38551,22 +38554,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
@@ -38660,7 +38663,7 @@
       <c r="B9" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="59">
+      <c r="C9" s="56">
         <v>139130.85</v>
       </c>
       <c r="D9" s="9" t="s">
@@ -38694,7 +38697,7 @@
       <c r="B11" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C11" s="60">
+      <c r="C11" s="57">
         <v>74.44</v>
       </c>
       <c r="D11" s="9" t="s">
@@ -39560,20 +39563,20 @@
         <v>4</v>
       </c>
       <c r="D3" s="49">
-        <f>concentration_risk!B4</f>
-        <v>1695</v>
+        <f>concentration_risk!B3</f>
+        <v>1473</v>
       </c>
       <c r="E3" s="25">
-        <f>concentration_risk!C4</f>
-        <v>24.07</v>
+        <f>concentration_risk!C3</f>
+        <v>20.91</v>
       </c>
       <c r="F3" s="38">
-        <f>concentration_risk!D4</f>
-        <v>103005.85</v>
+        <f>concentration_risk!D3</f>
+        <v>95816.6</v>
       </c>
       <c r="G3" s="55">
-        <f>concentration_risk!E4</f>
-        <v>22.58</v>
+        <f>concentration_risk!E3</f>
+        <v>21.01</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -39587,20 +39590,20 @@
         <v>5</v>
       </c>
       <c r="D4" s="48">
-        <f>concentration_risk!B3</f>
-        <v>1473</v>
+        <f>concentration_risk!B4</f>
+        <v>1695</v>
       </c>
       <c r="E4" s="35">
-        <f>concentration_risk!C3</f>
-        <v>20.91</v>
+        <f>concentration_risk!C4</f>
+        <v>24.07</v>
       </c>
       <c r="F4" s="36">
-        <f>concentration_risk!D3</f>
-        <v>95816.6</v>
+        <f>concentration_risk!D4</f>
+        <v>103005.85</v>
       </c>
       <c r="G4" s="54">
-        <f>concentration_risk!E3</f>
-        <v>21.01</v>
+        <f>concentration_risk!E4</f>
+        <v>22.58</v>
       </c>
     </row>
     <row r="6" spans="1:8">

</xml_diff>

<commit_message>
fix: link revenue KPI card to the percentage cell; ignore .DS_Store
</commit_message>
<xml_diff>
--- a/Telco_Churn_Analysis.xlsx
+++ b/Telco_Churn_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taofeeksalami/Telco_Customer_Churn_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B7A61C-3CF8-134F-8319-DDBBA78DA0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC24EA6-1DBB-AE45-A4F6-D22722C2DD57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="MKno8Rk8H3j9R42XnMw+0cJYymN9JmN8CmEIujZH0aKW3574fpr/rsIVHwELVCPliSOdVnIkew4dErdPTIs9BQ==" workbookSaltValue="XMxiKTKcD+NALzw573fuOQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14500" firstSheet="20" activeTab="24" xr2:uid="{B76D0E22-31AB-FB41-B59B-52BD901C65CA}"/>
@@ -32054,8 +32054,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="446617" y="486833"/>
-          <a:ext cx="736600" cy="685799"/>
+          <a:off x="446617" y="475544"/>
+          <a:ext cx="742244" cy="668866"/>
           <a:chOff x="853017" y="503766"/>
           <a:chExt cx="800100" cy="685799"/>
         </a:xfrm>
@@ -32481,8 +32481,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="444496" y="2983654"/>
-          <a:ext cx="736600" cy="640080"/>
+          <a:off x="444496" y="2904632"/>
+          <a:ext cx="742244" cy="623146"/>
           <a:chOff x="850900" y="2979669"/>
           <a:chExt cx="838200" cy="635598"/>
         </a:xfrm>
@@ -33570,8 +33570,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1820335" y="5530848"/>
-          <a:ext cx="14294303" cy="1839058"/>
+          <a:off x="1831624" y="5378448"/>
+          <a:ext cx="14390258" cy="1788258"/>
           <a:chOff x="1820335" y="8337548"/>
           <a:chExt cx="14294303" cy="1839058"/>
         </a:xfrm>
@@ -34347,7 +34347,7 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="KPI_Framework!C9">
+    <xdr:sp macro="" textlink="KPI_Framework!C10">
       <xdr:nvSpPr>
         <xdr:cNvPr id="50" name="Rounded Rectangle 49">
           <a:extLst>
@@ -34413,7 +34413,7 @@
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:pPr marL="0" indent="0" algn="l"/>
-            <a:t>£139,131</a:t>
+            <a:t>30.50%</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="3600" b="1">
             <a:solidFill>

</xml_diff>

<commit_message>
fix: correct swapped contract shares, a mislinked KPI card and dashboard wording (#3)
* fix: correct swapped contract shares and dashboard wording; relabel revenue lost to churn

* fix: link revenue KPI card to the percentage cell; ignore .DS_Store
</commit_message>
<xml_diff>
--- a/Telco_Churn_Analysis.xlsx
+++ b/Telco_Churn_Analysis.xlsx
@@ -5,13 +5,13 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taofeeksalami/Desktop/Harjii/DAV_Portfolio/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taofeeksalami/Telco_Customer_Churn_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B7A61C-3CF8-134F-8319-DDBBA78DA0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC24EA6-1DBB-AE45-A4F6-D22722C2DD57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="MKno8Rk8H3j9R42XnMw+0cJYymN9JmN8CmEIujZH0aKW3574fpr/rsIVHwELVCPliSOdVnIkew4dErdPTIs9BQ==" workbookSaltValue="XMxiKTKcD+NALzw573fuOQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16500" firstSheet="16" activeTab="24" xr2:uid="{B76D0E22-31AB-FB41-B59B-52BD901C65CA}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="14500" firstSheet="20" activeTab="24" xr2:uid="{B76D0E22-31AB-FB41-B59B-52BD901C65CA}"/>
   </bookViews>
   <sheets>
     <sheet name="perfect_storm_churn" sheetId="15" r:id="rId1"/>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="112">
   <si>
     <t>No</t>
   </si>
@@ -381,13 +381,13 @@
     <t>tbl_AvgTenureByChurn</t>
   </si>
   <si>
-    <t>Monthly Revenue at Risk (£)</t>
+    <t>Monthly Revenue Lost to Churn (£)</t>
   </si>
   <si>
     <t>tbl_RevenueAtRisk</t>
   </si>
   <si>
-    <t>Revenue at Risk %</t>
+    <t>Revenue Lost to Churn (% of monthly charges)</t>
   </si>
   <si>
     <t>Avg Monthly Charge — Churned (£)</t>
@@ -453,10 +453,10 @@
     <t>High Risk</t>
   </si>
   <si>
-    <t>Revenue at Risk Summary</t>
+    <t>Revenue Lost to Churn Summary</t>
   </si>
   <si>
-    <t>Annualised Revenue at Risk (£)</t>
+    <t>Annualised Revenue Lost to Churn (£)</t>
   </si>
   <si>
     <t>Project 7 — KPI Framework</t>
@@ -469,6 +469,9 @@
   </si>
   <si>
     <t>Segment Descriptions</t>
+  </si>
+  <si>
+    <t>Revenue Lost to Churn (% of monthly charges)</t>
   </si>
 </sst>
 </file>
@@ -712,6 +715,8 @@
     <xf numFmtId="2" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -721,8 +726,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2378,10 +2381,10 @@
                   <c:v>55.02</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.07</c:v>
+                  <c:v>20.91</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.91</c:v>
+                  <c:v>24.07</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2490,10 +2493,10 @@
                   <c:v>56.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.58</c:v>
+                  <c:v>21.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.01</c:v>
+                  <c:v>22.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5141,10 +5144,10 @@
                   <c:v>55.02</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.07</c:v>
+                  <c:v>20.91</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.91</c:v>
+                  <c:v>24.07</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5256,10 +5259,10 @@
                   <c:v>56.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.58</c:v>
+                  <c:v>21.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.01</c:v>
+                  <c:v>22.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7155,10 +7158,10 @@
                   <c:v>55.02</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.07</c:v>
+                  <c:v>20.91</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.91</c:v>
+                  <c:v>24.07</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7267,10 +7270,10 @@
                   <c:v>56.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22.58</c:v>
+                  <c:v>21.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21.01</c:v>
+                  <c:v>22.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8293,7 +8296,7 @@
                 </a:solidFill>
                 <a:effectLst/>
               </a:rPr>
-              <a:t>Monthly Revenue at Risk vs Retained</a:t>
+              <a:t>Monthly Revenue Lost vs Retained</a:t>
             </a:r>
             <a:endParaRPr lang="en-GB" sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -24910,7 +24913,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Month-to-month contracts are the strongest churn driver (42.71%), with a churn rate 15× higher than two-year contracts.</a:t>
+            <a:t>• Month-to-month contracts have the highest churn rate (42.71%), 15× that of two-year contracts.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -24922,7 +24925,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Customer attrition is concentrated early, with 47.44% of churn occurring within the first 12 months.</a:t>
+            <a:t>• Churn is concentrated early: customers in their first 12 months churn at 47.44% and make up 55.5% of all churners.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -24934,7 +24937,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Electronic check customers are the highest-risk payment segment, with a churn rate of 45.29%—more than 3× that of automatic payment customers.</a:t>
+            <a:t>• Electronic check customers have the highest churn rate of any payment method (45.29%), about 3× that of automatic payment (15.2–16.7%).</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -25618,7 +25621,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>⚠ Early tenure churn</a:t>
+            <a:t>⚠ 0–12 month churn rate</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27010,7 +27013,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Customer Churn Puts £1.67M of Annual Revenue at Risk</a:t>
+            <a:t>Churned Customers Were Paying £1.67M a Year</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27290,7 +27293,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Month-to-month customers record the highest churn rate (42.7%) while also representing the largest share of monthly revenue exposure.</a:t>
+            <a:t>Month-to-month customers record the highest churn rate (42.7%) while also contributing the largest share of monthly revenue (56.4%).</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27545,7 +27548,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue at risk</a:t>
+            <a:t>Revenue lost to churn</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -27997,7 +28000,7 @@
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>Monthly Revenue at Risk vs Retained</a:t>
+              <a:t>Monthly Revenue Lost vs Retained</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -28394,7 +28397,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Month-to-month contracts are the primary churn driver, with a churn rate of 42.71%—15× higher than two-year contracts.</a:t>
+            <a:t>• Month-to-month contracts have the highest churn rate, 42.71%—15× that of two-year contracts.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -28406,7 +28409,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Current churn represents a monthly revenue loss of £139K (30.5%), placing an estimated £1.67M in annual revenue at risk.</a:t>
+            <a:t>• Churned customers had been paying £139K a month (30.5% of monthly charges), about £1.67M a year.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -28418,7 +28421,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• A cohort of 814 high-risk customers is churning at 69.53%—more than three times the standard customer churn rate (20.92%).</a:t>
+            <a:t>• 814 customers fit the high-risk profile and churned at 69.53%, 3.3× the 20.92% rate for all others; 566 had already left.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -28646,7 +28649,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>• Target the 814 high-risk customers with personalised retention offers before renewal.</a:t>
+            <a:t>• Test the high-risk profile on active customers before using it to target offers.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -31066,7 +31069,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• The business is heavily exposed to month-to-month contracts, where 55% of customers generate 56% of total revenue.</a:t>
+              <a:t>• The business is heavily exposed to month-to-month contracts, where 55% of customers generate 56% of monthly revenue.</a:t>
             </a:r>
           </a:p>
           <a:p>
@@ -31090,7 +31093,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• The 814 high-risk customers are churning at 69.53%—more than three times the rate of the standard customer base (20.92%).</a:t>
+              <a:t>• The 814 customers in the high-risk profile churned at 69.53%, 3.3× the 20.92% rate for all others; 566 had already left.</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -31285,7 +31288,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• Implement proactive outreach for high-risk customers using early-warning indicators and personalised retention offers.</a:t>
+              <a:t>• Test the high-risk profile on active customers; if it holds, use it to prioritise outreach and retention offers.</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -32051,8 +32054,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="446617" y="486833"/>
-          <a:ext cx="736600" cy="685799"/>
+          <a:off x="446617" y="475544"/>
+          <a:ext cx="742244" cy="668866"/>
           <a:chOff x="853017" y="503766"/>
           <a:chExt cx="800100" cy="685799"/>
         </a:xfrm>
@@ -32478,8 +32481,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="444496" y="2983654"/>
-          <a:ext cx="736600" cy="640080"/>
+          <a:off x="444496" y="2904632"/>
+          <a:ext cx="742244" cy="623146"/>
           <a:chOff x="850900" y="2979669"/>
           <a:chExt cx="838200" cy="635598"/>
         </a:xfrm>
@@ -33193,7 +33196,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue Stability Analysis — At Risk Revenue, Contract Value &amp; Customer LTV</a:t>
+            <a:t>Revenue Stability Analysis — Revenue Lost to Churn, Contract Value &amp; Customer LTV</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -33269,7 +33272,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue pillar · Total monthly charges £456K · 30.5% at risk · Annualised risk £1.67M</a:t>
+            <a:t>Revenue pillar · Total monthly charges £456K · 30.5% lost to churn · £1.67M a year</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -33496,7 +33499,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Monthly Revenue at Risk vs Retained</a:t>
+            <a:t>Monthly Revenue Lost vs Retained</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -33567,8 +33570,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1820335" y="5530848"/>
-          <a:ext cx="14294303" cy="1839058"/>
+          <a:off x="1831624" y="5378448"/>
+          <a:ext cx="14390258" cy="1788258"/>
           <a:chOff x="1820335" y="8337548"/>
           <a:chExt cx="14294303" cy="1839058"/>
         </a:xfrm>
@@ -33738,7 +33741,7 @@
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>• The business is losing its highest-value customers, with churned customers paying £13.17 more per month on average than retained customers.</a:t>
+              <a:t>• Churned customers were paying £13.17 more per month on average than retained customers (£74.44 vs £61.27).</a:t>
             </a:r>
           </a:p>
           <a:p>
@@ -34344,7 +34347,7 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="KPI_Framework!C9">
+    <xdr:sp macro="" textlink="KPI_Framework!C10">
       <xdr:nvSpPr>
         <xdr:cNvPr id="50" name="Rounded Rectangle 49">
           <a:extLst>
@@ -34460,7 +34463,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Revenue at risk</a:t>
+            <a:t>Revenue lost to churn</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -37123,10 +37126,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="58" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="56"/>
+      <c r="B1" s="58"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
@@ -37169,7 +37172,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="27" t="s">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="B5" s="29">
         <f>revenue_at_risk!D2</f>
@@ -38551,22 +38554,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
@@ -38660,7 +38663,7 @@
       <c r="B9" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="59">
+      <c r="C9" s="56">
         <v>139130.85</v>
       </c>
       <c r="D9" s="9" t="s">
@@ -38694,7 +38697,7 @@
       <c r="B11" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C11" s="60">
+      <c r="C11" s="57">
         <v>74.44</v>
       </c>
       <c r="D11" s="9" t="s">
@@ -39560,20 +39563,20 @@
         <v>4</v>
       </c>
       <c r="D3" s="49">
-        <f>concentration_risk!B4</f>
-        <v>1695</v>
+        <f>concentration_risk!B3</f>
+        <v>1473</v>
       </c>
       <c r="E3" s="25">
-        <f>concentration_risk!C4</f>
-        <v>24.07</v>
+        <f>concentration_risk!C3</f>
+        <v>20.91</v>
       </c>
       <c r="F3" s="38">
-        <f>concentration_risk!D4</f>
-        <v>103005.85</v>
+        <f>concentration_risk!D3</f>
+        <v>95816.6</v>
       </c>
       <c r="G3" s="55">
-        <f>concentration_risk!E4</f>
-        <v>22.58</v>
+        <f>concentration_risk!E3</f>
+        <v>21.01</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -39587,20 +39590,20 @@
         <v>5</v>
       </c>
       <c r="D4" s="48">
-        <f>concentration_risk!B3</f>
-        <v>1473</v>
+        <f>concentration_risk!B4</f>
+        <v>1695</v>
       </c>
       <c r="E4" s="35">
-        <f>concentration_risk!C3</f>
-        <v>20.91</v>
+        <f>concentration_risk!C4</f>
+        <v>24.07</v>
       </c>
       <c r="F4" s="36">
-        <f>concentration_risk!D3</f>
-        <v>95816.6</v>
+        <f>concentration_risk!D4</f>
+        <v>103005.85</v>
       </c>
       <c r="G4" s="54">
-        <f>concentration_risk!E3</f>
-        <v>21.01</v>
+        <f>concentration_risk!E4</f>
+        <v>22.58</v>
       </c>
     </row>
     <row r="6" spans="1:8">

</xml_diff>